<commit_message>
state: session end 2026-08-24T10:04Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS66"/>
+  <dimension ref="A1:AS67"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8361,9 +8361,146 @@
         <v>bias Bearish persisted 1/3 polls</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-08-24 15:30:30</v>
+      </c>
+      <c r="B67">
+        <v>77370.13</v>
+      </c>
+      <c r="C67">
+        <v>77400</v>
+      </c>
+      <c r="D67">
+        <v>0.77</v>
+      </c>
+      <c r="E67">
+        <v>75500</v>
+      </c>
+      <c r="F67">
+        <v>77500</v>
+      </c>
+      <c r="G67">
+        <v>77300</v>
+      </c>
+      <c r="H67">
+        <v>77500</v>
+      </c>
+      <c r="I67">
+        <v>78000</v>
+      </c>
+      <c r="J67">
+        <v>77700</v>
+      </c>
+      <c r="K67">
+        <v>29</v>
+      </c>
+      <c r="L67">
+        <v>41</v>
+      </c>
+      <c r="M67">
+        <v>3315300</v>
+      </c>
+      <c r="N67">
+        <v>4556940</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Put Covering 9x/582480 | Put Buying 23x/2167360 | Call Buying 23x/3254400 | Call Writing 9x/1807100 | Call Covering 3x/48560 | Put Writing 2x/12040 | Put Unwinding 1x/300</v>
+      </c>
+      <c r="P67">
+        <v>11.86</v>
+      </c>
+      <c r="Q67" t="str">
+        <v>Range</v>
+      </c>
+      <c r="R67">
+        <v>0.518</v>
+      </c>
+      <c r="S67">
+        <v>0.484</v>
+      </c>
+      <c r="T67">
+        <v>29.659</v>
+      </c>
+      <c r="U67">
+        <v>0.0003</v>
+      </c>
+      <c r="V67">
+        <v>14.698</v>
+      </c>
+      <c r="W67" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X67">
+        <v>77596.72</v>
+      </c>
+      <c r="Y67">
+        <v>0.66</v>
+      </c>
+      <c r="Z67" t="str">
+        <v>Neutral</v>
+      </c>
+      <c r="AA67">
+        <v>83</v>
+      </c>
+      <c r="AB67" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AC67">
+        <v>75</v>
+      </c>
+      <c r="AD67" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE67">
+        <v>70</v>
+      </c>
+      <c r="AF67" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AG67">
+        <v>30</v>
+      </c>
+      <c r="AH67">
+        <v>50000</v>
+      </c>
+      <c r="AI67" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AJ67" t="str">
+        <v>BUY 77400PE | SELL 77300PE</v>
+      </c>
+      <c r="AK67">
+        <v>1</v>
+      </c>
+      <c r="AL67">
+        <v>41.95</v>
+      </c>
+      <c r="AM67">
+        <v>20.98</v>
+      </c>
+      <c r="AN67">
+        <v>83.9</v>
+      </c>
+      <c r="AO67">
+        <v>420</v>
+      </c>
+      <c r="AP67">
+        <v>839</v>
+      </c>
+      <c r="AQ67">
+        <v>2</v>
+      </c>
+      <c r="AR67" t="str">
+        <v>default</v>
+      </c>
+      <c r="AS67" t="str">
+        <v>bias Range persisted 1/3 polls</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS67"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-26T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -23001,7 +23001,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS55"/>
+  <dimension ref="A1:AS57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -29788,9 +29788,253 @@
         <v>bias Bearish persisted 1/3 polls</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>2026-08-26 12:31:57</v>
+      </c>
+      <c r="B56">
+        <v>77657.13</v>
+      </c>
+      <c r="C56">
+        <v>77700</v>
+      </c>
+      <c r="D56">
+        <v>0.7</v>
+      </c>
+      <c r="E56">
+        <v>77500</v>
+      </c>
+      <c r="F56">
+        <v>77700</v>
+      </c>
+      <c r="G56">
+        <v>77600</v>
+      </c>
+      <c r="H56">
+        <v>78000</v>
+      </c>
+      <c r="I56">
+        <v>77800</v>
+      </c>
+      <c r="J56">
+        <v>77900</v>
+      </c>
+      <c r="K56">
+        <v>22</v>
+      </c>
+      <c r="L56">
+        <v>47</v>
+      </c>
+      <c r="M56">
+        <v>12616600</v>
+      </c>
+      <c r="N56">
+        <v>34281460</v>
+      </c>
+      <c r="O56" t="str">
+        <v>Put Writing 10x/4042240 | Call Writing 15x/23491140 | Call Unwinding 10x/247080 | Put Unwinding 1x/281680 | Put Buying 21x/10542840 | Call Buying 11x/8292680 | Put Covering 1x/400</v>
+      </c>
+      <c r="P56">
+        <v>13.41</v>
+      </c>
+      <c r="Q56" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R56">
+        <v>0.501</v>
+      </c>
+      <c r="S56">
+        <v>0.497</v>
+      </c>
+      <c r="T56">
+        <v>39.272</v>
+      </c>
+      <c r="U56">
+        <v>0.0003</v>
+      </c>
+      <c r="V56">
+        <v>6.552</v>
+      </c>
+      <c r="W56" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X56">
+        <v>77962.64</v>
+      </c>
+      <c r="Y56">
+        <v>0.1</v>
+      </c>
+      <c r="Z56" t="str">
+        <v>Long Unwinding</v>
+      </c>
+      <c r="AA56">
+        <v>83</v>
+      </c>
+      <c r="AB56" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AC56">
+        <v>100</v>
+      </c>
+      <c r="AD56" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE56">
+        <v>70</v>
+      </c>
+      <c r="AF56" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AG56">
+        <v>60</v>
+      </c>
+      <c r="AH56">
+        <v>50000</v>
+      </c>
+      <c r="AI56" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AJ56" t="str">
+        <v>BUY 77700PE | SELL 77600PE</v>
+      </c>
+      <c r="AK56">
+        <v>1</v>
+      </c>
+      <c r="AL56">
+        <v>38.55</v>
+      </c>
+      <c r="AM56">
+        <v>19.28</v>
+      </c>
+      <c r="AN56" t="str">
+        <v>SIGNAL</v>
+      </c>
+      <c r="AO56">
+        <v>386</v>
+      </c>
+      <c r="AP56" t="str">
+        <v/>
+      </c>
+      <c r="AQ56" t="str">
+        <v/>
+      </c>
+      <c r="AR56" t="str">
+        <v>ride</v>
+      </c>
+      <c r="AS56" t="str">
+        <v>bias Bearish persisted 2/3 polls</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>2026-08-26 12:34:57</v>
+      </c>
+      <c r="B57">
+        <v>77668.46</v>
+      </c>
+      <c r="C57">
+        <v>77700</v>
+      </c>
+      <c r="D57">
+        <v>0.69</v>
+      </c>
+      <c r="E57">
+        <v>77500</v>
+      </c>
+      <c r="F57">
+        <v>77700</v>
+      </c>
+      <c r="G57">
+        <v>77600</v>
+      </c>
+      <c r="H57">
+        <v>78000</v>
+      </c>
+      <c r="I57">
+        <v>77800</v>
+      </c>
+      <c r="J57">
+        <v>77900</v>
+      </c>
+      <c r="K57">
+        <v>52</v>
+      </c>
+      <c r="L57">
+        <v>16</v>
+      </c>
+      <c r="M57">
+        <v>40573600</v>
+      </c>
+      <c r="N57">
+        <v>7519900</v>
+      </c>
+      <c r="O57" t="str">
+        <v>Put Buying 2x/82600 | Call Writing 11x/7430420 | Call Unwinding 2x/6480 | Put Writing 28x/14523100 | Call Covering 8x/233240 | Put Unwinding 1x/268940 | Call Buying 15x/25548320 | Put Covering 1x/400</v>
+      </c>
+      <c r="P57">
+        <v>12.56</v>
+      </c>
+      <c r="Q57" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R57">
+        <v>0.495</v>
+      </c>
+      <c r="S57">
+        <v>0.507</v>
+      </c>
+      <c r="T57">
+        <v>38.692</v>
+      </c>
+      <c r="U57">
+        <v>0.0003</v>
+      </c>
+      <c r="V57">
+        <v>6.275</v>
+      </c>
+      <c r="W57" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X57">
+        <v>77962.64</v>
+      </c>
+      <c r="Y57">
+        <v>0.1</v>
+      </c>
+      <c r="Z57" t="str">
+        <v>Neutral</v>
+      </c>
+      <c r="AA57">
+        <v>67</v>
+      </c>
+      <c r="AB57" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AC57">
+        <v>75</v>
+      </c>
+      <c r="AD57" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE57">
+        <v>70</v>
+      </c>
+      <c r="AF57" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AG57">
+        <v>60</v>
+      </c>
+      <c r="AH57">
+        <v>50000</v>
+      </c>
+      <c r="AI57" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-28T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -42788,7 +42788,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS66"/>
+  <dimension ref="A1:AS67"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -50152,9 +50152,116 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-08-28 12:32:31</v>
+      </c>
+      <c r="B67">
+        <v>77063.24</v>
+      </c>
+      <c r="C67">
+        <v>77100</v>
+      </c>
+      <c r="D67">
+        <v>0.83</v>
+      </c>
+      <c r="E67">
+        <v>77000</v>
+      </c>
+      <c r="F67">
+        <v>77100</v>
+      </c>
+      <c r="G67">
+        <v>77500</v>
+      </c>
+      <c r="H67">
+        <v>77500</v>
+      </c>
+      <c r="I67">
+        <v>78000</v>
+      </c>
+      <c r="J67">
+        <v>77300</v>
+      </c>
+      <c r="K67">
+        <v>67</v>
+      </c>
+      <c r="L67">
+        <v>2</v>
+      </c>
+      <c r="M67">
+        <v>9888580</v>
+      </c>
+      <c r="N67">
+        <v>60220</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Put Writing 37x/4387180 | Call Buying 30x/5501400 | Call Writing 1x/60060 | Put Buying 1x/160</v>
+      </c>
+      <c r="P67">
+        <v>10.22</v>
+      </c>
+      <c r="Q67" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R67">
+        <v>0.511</v>
+      </c>
+      <c r="S67">
+        <v>0.491</v>
+      </c>
+      <c r="T67">
+        <v>22.358</v>
+      </c>
+      <c r="U67">
+        <v>0.0002</v>
+      </c>
+      <c r="V67">
+        <v>24.497</v>
+      </c>
+      <c r="W67" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X67">
+        <v>77867.43</v>
+      </c>
+      <c r="Y67">
+        <v>0.13</v>
+      </c>
+      <c r="Z67" t="str">
+        <v>Neutral</v>
+      </c>
+      <c r="AA67">
+        <v>67</v>
+      </c>
+      <c r="AB67" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AC67">
+        <v>75</v>
+      </c>
+      <c r="AD67" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE67">
+        <v>70</v>
+      </c>
+      <c r="AF67" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AG67">
+        <v>60</v>
+      </c>
+      <c r="AH67">
+        <v>50000</v>
+      </c>
+      <c r="AI67" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS67"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-31T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -50269,7 +50269,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS48"/>
+  <dimension ref="A1:AS49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -55977,9 +55977,116 @@
         <v>bias Bullish persisted 1/3 polls</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>2026-08-31 12:32:22</v>
+      </c>
+      <c r="B49">
+        <v>76960.53</v>
+      </c>
+      <c r="C49">
+        <v>77000</v>
+      </c>
+      <c r="D49">
+        <v>1.14</v>
+      </c>
+      <c r="E49">
+        <v>77000</v>
+      </c>
+      <c r="F49">
+        <v>75000</v>
+      </c>
+      <c r="G49">
+        <v>76800</v>
+      </c>
+      <c r="H49">
+        <v>77000</v>
+      </c>
+      <c r="I49">
+        <v>78000</v>
+      </c>
+      <c r="J49">
+        <v>77500</v>
+      </c>
+      <c r="K49">
+        <v>8</v>
+      </c>
+      <c r="L49">
+        <v>59</v>
+      </c>
+      <c r="M49">
+        <v>384120</v>
+      </c>
+      <c r="N49">
+        <v>9186840</v>
+      </c>
+      <c r="O49" t="str">
+        <v>Put Writing 8x/384120 | Call Writing 31x/4481860 | Put Buying 23x/4500760 | Put Covering 4x/168820 | Call Unwinding 1x/35400</v>
+      </c>
+      <c r="P49">
+        <v>12.56</v>
+      </c>
+      <c r="Q49" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R49">
+        <v>0.489</v>
+      </c>
+      <c r="S49">
+        <v>0.521</v>
+      </c>
+      <c r="T49">
+        <v>38.101</v>
+      </c>
+      <c r="U49">
+        <v>0.0002</v>
+      </c>
+      <c r="V49">
+        <v>15.713</v>
+      </c>
+      <c r="W49" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X49">
+        <v>77535.77</v>
+      </c>
+      <c r="Y49">
+        <v>0.08</v>
+      </c>
+      <c r="Z49" t="str">
+        <v>Neutral</v>
+      </c>
+      <c r="AA49">
+        <v>67</v>
+      </c>
+      <c r="AB49" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AC49">
+        <v>75</v>
+      </c>
+      <c r="AD49" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE49">
+        <v>70</v>
+      </c>
+      <c r="AF49" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AG49">
+        <v>60</v>
+      </c>
+      <c r="AH49">
+        <v>50000</v>
+      </c>
+      <c r="AI49" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-09-02T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -725,7 +725,7 @@
         <v>2026-09-02 12:03:43</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>2026-09-02 12:33:43</v>
       </c>
       <c r="D6" t="str">
         <v>intraday</v>
@@ -745,23 +745,23 @@
       <c r="I6">
         <v>43.5</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
+      <c r="J6">
+        <v>35.1</v>
       </c>
       <c r="K6" t="str">
-        <v>OPEN</v>
+        <v>LOSS</v>
       </c>
       <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
-        <v/>
+        <v>SIGNAL_CHANGE</v>
+      </c>
+      <c r="M6">
+        <v>-168</v>
       </c>
       <c r="N6">
         <v>110.31</v>
       </c>
-      <c r="O6" t="str">
-        <v/>
+      <c r="O6">
+        <v>-278.31</v>
       </c>
       <c r="P6" t="str">
         <v>ride</v>
@@ -63413,7 +63413,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS66"/>
+  <dimension ref="A1:AS68"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -71617,9 +71617,253 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-09-02 12:30:43</v>
+      </c>
+      <c r="B67">
+        <v>76343.68</v>
+      </c>
+      <c r="C67">
+        <v>76300</v>
+      </c>
+      <c r="D67">
+        <v>0.76</v>
+      </c>
+      <c r="E67">
+        <v>76000</v>
+      </c>
+      <c r="F67">
+        <v>76200</v>
+      </c>
+      <c r="G67">
+        <v>76300</v>
+      </c>
+      <c r="H67">
+        <v>77000</v>
+      </c>
+      <c r="I67">
+        <v>76500</v>
+      </c>
+      <c r="J67">
+        <v>77500</v>
+      </c>
+      <c r="K67">
+        <v>60</v>
+      </c>
+      <c r="L67">
+        <v>12</v>
+      </c>
+      <c r="M67">
+        <v>47493280</v>
+      </c>
+      <c r="N67">
+        <v>4404780</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Put Buying 4x/1126960 | Call Buying 27x/26763820 | Put Writing 21x/19797560 | Put Unwinding 12x/931900 | Call Writing 7x/3268960 | Call Unwinding 1x/8860</v>
+      </c>
+      <c r="P67">
+        <v>15.43</v>
+      </c>
+      <c r="Q67" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R67">
+        <v>0.495</v>
+      </c>
+      <c r="S67">
+        <v>0.503</v>
+      </c>
+      <c r="T67">
+        <v>60.387</v>
+      </c>
+      <c r="U67">
+        <v>0.0002</v>
+      </c>
+      <c r="V67">
+        <v>7.322</v>
+      </c>
+      <c r="W67" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X67">
+        <v>76850.02</v>
+      </c>
+      <c r="Y67">
+        <v>0.21</v>
+      </c>
+      <c r="Z67" t="str">
+        <v>Long Unwinding</v>
+      </c>
+      <c r="AA67">
+        <v>67</v>
+      </c>
+      <c r="AB67" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AC67">
+        <v>75</v>
+      </c>
+      <c r="AD67" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AE67">
+        <v>60</v>
+      </c>
+      <c r="AF67" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG67">
+        <v>50</v>
+      </c>
+      <c r="AH67">
+        <v>50000</v>
+      </c>
+      <c r="AI67" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2026-09-02 12:33:43</v>
+      </c>
+      <c r="B68">
+        <v>76379.64</v>
+      </c>
+      <c r="C68">
+        <v>76400</v>
+      </c>
+      <c r="D68">
+        <v>0.77</v>
+      </c>
+      <c r="E68">
+        <v>76000</v>
+      </c>
+      <c r="F68">
+        <v>76200</v>
+      </c>
+      <c r="G68">
+        <v>76300</v>
+      </c>
+      <c r="H68">
+        <v>77000</v>
+      </c>
+      <c r="I68">
+        <v>76500</v>
+      </c>
+      <c r="J68">
+        <v>77500</v>
+      </c>
+      <c r="K68">
+        <v>66</v>
+      </c>
+      <c r="L68">
+        <v>7</v>
+      </c>
+      <c r="M68">
+        <v>48688020</v>
+      </c>
+      <c r="N68">
+        <v>1587620</v>
+      </c>
+      <c r="O68" t="str">
+        <v>Put Buying 5x/1415420 | Put Writing 19x/19383120 | Call Buying 32x/28388300 | Put Unwinding 14x/908520 | Call Covering 1x/8080 | Call Writing 1x/171840 | Put Covering 1x/360</v>
+      </c>
+      <c r="P68">
+        <v>15.89</v>
+      </c>
+      <c r="Q68" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R68">
+        <v>0.485</v>
+      </c>
+      <c r="S68">
+        <v>0.513</v>
+      </c>
+      <c r="T68">
+        <v>61.85</v>
+      </c>
+      <c r="U68">
+        <v>0.0002</v>
+      </c>
+      <c r="V68">
+        <v>7.392</v>
+      </c>
+      <c r="W68" t="str">
+        <v>Up</v>
+      </c>
+      <c r="X68">
+        <v>76852.72</v>
+      </c>
+      <c r="Y68">
+        <v>1.43</v>
+      </c>
+      <c r="Z68" t="str">
+        <v>Short Covering</v>
+      </c>
+      <c r="AA68">
+        <v>83</v>
+      </c>
+      <c r="AB68" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AC68">
+        <v>100</v>
+      </c>
+      <c r="AD68" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AE68">
+        <v>75</v>
+      </c>
+      <c r="AF68" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG68">
+        <v>50</v>
+      </c>
+      <c r="AH68">
+        <v>50000</v>
+      </c>
+      <c r="AI68" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AJ68" t="str">
+        <v>BUY 76400CE | SELL 76500CE</v>
+      </c>
+      <c r="AK68">
+        <v>1</v>
+      </c>
+      <c r="AL68">
+        <v>51.05</v>
+      </c>
+      <c r="AM68">
+        <v>25.53</v>
+      </c>
+      <c r="AN68" t="str">
+        <v>SIGNAL</v>
+      </c>
+      <c r="AO68">
+        <v>511</v>
+      </c>
+      <c r="AP68" t="str">
+        <v/>
+      </c>
+      <c r="AQ68" t="str">
+        <v/>
+      </c>
+      <c r="AR68" t="str">
+        <v>ride</v>
+      </c>
+      <c r="AS68" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS68"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-09-03T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -789,7 +789,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS66"/>
+  <dimension ref="A1:AS68"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8123,9 +8123,223 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-09-03 12:31:11</v>
+      </c>
+      <c r="B67">
+        <v>76599.27</v>
+      </c>
+      <c r="C67">
+        <v>76600</v>
+      </c>
+      <c r="D67">
+        <v>0.85</v>
+      </c>
+      <c r="E67">
+        <v>77000</v>
+      </c>
+      <c r="F67">
+        <v>75000</v>
+      </c>
+      <c r="G67">
+        <v>76500</v>
+      </c>
+      <c r="H67">
+        <v>77000</v>
+      </c>
+      <c r="I67">
+        <v>78000</v>
+      </c>
+      <c r="J67">
+        <v>78500</v>
+      </c>
+      <c r="K67">
+        <v>44</v>
+      </c>
+      <c r="L67">
+        <v>14</v>
+      </c>
+      <c r="M67">
+        <v>1305820</v>
+      </c>
+      <c r="N67">
+        <v>199440</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Put Unwinding 2x/17000 | Put Writing 25x/715120 | Put Buying 4x/26580 | Call Buying 16x/573120 | Call Unwinding 2x/1040 | Call Writing 8x/171820 | Call Covering 1x/580</v>
+      </c>
+      <c r="P67">
+        <v>9.54</v>
+      </c>
+      <c r="Q67" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R67">
+        <v>0.545</v>
+      </c>
+      <c r="S67">
+        <v>0.485</v>
+      </c>
+      <c r="T67">
+        <v>20.477</v>
+      </c>
+      <c r="U67">
+        <v>0.0002</v>
+      </c>
+      <c r="V67">
+        <v>26.339</v>
+      </c>
+      <c r="W67" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X67">
+        <v>77231.62</v>
+      </c>
+      <c r="Y67">
+        <v>0.81</v>
+      </c>
+      <c r="Z67" t="str">
+        <v>Long Buildup</v>
+      </c>
+      <c r="AA67">
+        <v>50</v>
+      </c>
+      <c r="AB67" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AC67">
+        <v>75</v>
+      </c>
+      <c r="AD67" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE67">
+        <v>70</v>
+      </c>
+      <c r="AF67" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AG67">
+        <v>60</v>
+      </c>
+      <c r="AH67">
+        <v>50000</v>
+      </c>
+      <c r="AI67" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2026-09-03 12:34:13</v>
+      </c>
+      <c r="B68">
+        <v>76593.6</v>
+      </c>
+      <c r="C68">
+        <v>76600</v>
+      </c>
+      <c r="D68">
+        <v>0.85</v>
+      </c>
+      <c r="E68">
+        <v>77000</v>
+      </c>
+      <c r="F68">
+        <v>76500</v>
+      </c>
+      <c r="G68">
+        <v>75000</v>
+      </c>
+      <c r="H68">
+        <v>77000</v>
+      </c>
+      <c r="I68">
+        <v>78000</v>
+      </c>
+      <c r="J68">
+        <v>78500</v>
+      </c>
+      <c r="K68">
+        <v>25</v>
+      </c>
+      <c r="L68">
+        <v>35</v>
+      </c>
+      <c r="M68">
+        <v>344520</v>
+      </c>
+      <c r="N68">
+        <v>1177820</v>
+      </c>
+      <c r="O68" t="str">
+        <v>Put Covering 2x/18060 | Put Buying 17x/585420 | Put Writing 12x/141660 | Call Buying 11x/201820 | Call Writing 15x/574260 | Call Covering 2x/1040 | Call Unwinding 1x/80</v>
+      </c>
+      <c r="P68">
+        <v>9.58</v>
+      </c>
+      <c r="Q68" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R68">
+        <v>0.544</v>
+      </c>
+      <c r="S68">
+        <v>0.485</v>
+      </c>
+      <c r="T68">
+        <v>20.63</v>
+      </c>
+      <c r="U68">
+        <v>0.0002</v>
+      </c>
+      <c r="V68">
+        <v>26.41</v>
+      </c>
+      <c r="W68" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X68">
+        <v>77229.2</v>
+      </c>
+      <c r="Y68">
+        <v>0.53</v>
+      </c>
+      <c r="Z68" t="str">
+        <v>Long Buildup</v>
+      </c>
+      <c r="AA68">
+        <v>67</v>
+      </c>
+      <c r="AB68" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AC68">
+        <v>100</v>
+      </c>
+      <c r="AD68" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE68">
+        <v>70</v>
+      </c>
+      <c r="AF68" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AG68">
+        <v>40</v>
+      </c>
+      <c r="AH68">
+        <v>50000</v>
+      </c>
+      <c r="AI68" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS68"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
state: session end 2026-09-04T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -12518,7 +12518,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS62"/>
+  <dimension ref="A1:AS64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20264,9 +20264,223 @@
         <v>bias Bullish persisted 1/3 polls</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-09-04 12:31:30</v>
+      </c>
+      <c r="B63">
+        <v>76719.72</v>
+      </c>
+      <c r="C63">
+        <v>76700</v>
+      </c>
+      <c r="D63">
+        <v>1.26</v>
+      </c>
+      <c r="E63">
+        <v>76500</v>
+      </c>
+      <c r="F63">
+        <v>76700</v>
+      </c>
+      <c r="G63">
+        <v>76600</v>
+      </c>
+      <c r="H63">
+        <v>77000</v>
+      </c>
+      <c r="I63">
+        <v>78000</v>
+      </c>
+      <c r="J63">
+        <v>76800</v>
+      </c>
+      <c r="K63">
+        <v>7</v>
+      </c>
+      <c r="L63">
+        <v>58</v>
+      </c>
+      <c r="M63">
+        <v>308900</v>
+      </c>
+      <c r="N63">
+        <v>11632440</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Put Buying 32x/7627080 | Call Writing 26x/4005360 | Call Buying 4x/296200 | Put Writing 3x/12700</v>
+      </c>
+      <c r="P63">
+        <v>10.98</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R63">
+        <v>0.526</v>
+      </c>
+      <c r="S63">
+        <v>0.473</v>
+      </c>
+      <c r="T63">
+        <v>22.946</v>
+      </c>
+      <c r="U63">
+        <v>0.0002</v>
+      </c>
+      <c r="V63">
+        <v>25.255</v>
+      </c>
+      <c r="W63" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X63">
+        <v>77103.43</v>
+      </c>
+      <c r="Y63">
+        <v>0.4</v>
+      </c>
+      <c r="Z63" t="str">
+        <v>Neutral</v>
+      </c>
+      <c r="AA63">
+        <v>67</v>
+      </c>
+      <c r="AB63" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AC63">
+        <v>75</v>
+      </c>
+      <c r="AD63" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE63">
+        <v>70</v>
+      </c>
+      <c r="AF63" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AG63">
+        <v>60</v>
+      </c>
+      <c r="AH63">
+        <v>50000</v>
+      </c>
+      <c r="AI63" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2026-09-04 12:34:30</v>
+      </c>
+      <c r="B64">
+        <v>76714.18</v>
+      </c>
+      <c r="C64">
+        <v>76700</v>
+      </c>
+      <c r="D64">
+        <v>1.25</v>
+      </c>
+      <c r="E64">
+        <v>76500</v>
+      </c>
+      <c r="F64">
+        <v>76700</v>
+      </c>
+      <c r="G64">
+        <v>76600</v>
+      </c>
+      <c r="H64">
+        <v>77000</v>
+      </c>
+      <c r="I64">
+        <v>78000</v>
+      </c>
+      <c r="J64">
+        <v>76800</v>
+      </c>
+      <c r="K64">
+        <v>8</v>
+      </c>
+      <c r="L64">
+        <v>56</v>
+      </c>
+      <c r="M64">
+        <v>132340</v>
+      </c>
+      <c r="N64">
+        <v>12023480</v>
+      </c>
+      <c r="O64" t="str">
+        <v>Put Buying 30x/7552620 | Put Writing 4x/97120 | Call Buying 4x/35220 | Call Writing 26x/4470860</v>
+      </c>
+      <c r="P64">
+        <v>11.02</v>
+      </c>
+      <c r="Q64" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R64">
+        <v>0.521</v>
+      </c>
+      <c r="S64">
+        <v>0.476</v>
+      </c>
+      <c r="T64">
+        <v>23.087</v>
+      </c>
+      <c r="U64">
+        <v>0.0002</v>
+      </c>
+      <c r="V64">
+        <v>25.345</v>
+      </c>
+      <c r="W64" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X64">
+        <v>77103.38</v>
+      </c>
+      <c r="Y64">
+        <v>0.2</v>
+      </c>
+      <c r="Z64" t="str">
+        <v>Short Buildup</v>
+      </c>
+      <c r="AA64">
+        <v>67</v>
+      </c>
+      <c r="AB64" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AC64">
+        <v>75</v>
+      </c>
+      <c r="AD64" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AE64">
+        <v>70</v>
+      </c>
+      <c r="AF64" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AG64">
+        <v>60</v>
+      </c>
+      <c r="AH64">
+        <v>50000</v>
+      </c>
+      <c r="AI64" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS64"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>